<commit_message>
feat: add sum total in export
</commit_message>
<xml_diff>
--- a/public/assets/templates/utility/laporan_air_utility.xlsx
+++ b/public/assets/templates/utility/laporan_air_utility.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\utility\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3D91BB2-02CC-47C5-B70E-C7436F914F84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C403ED4F-C85D-4293-ADB8-3DCECD69851C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{99CC749A-043A-42C9-9CA5-3CA614D07719}"/>
   </bookViews>
@@ -582,15 +582,69 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -609,67 +663,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1103,173 +1103,173 @@
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="47" t="s">
+      <c r="D1" s="39" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-      <c r="H1" s="48"/>
-      <c r="I1" s="48"/>
-      <c r="J1" s="48"/>
-      <c r="K1" s="48"/>
-      <c r="L1" s="48"/>
-      <c r="M1" s="48"/>
-      <c r="N1" s="48"/>
-      <c r="O1" s="48"/>
-      <c r="P1" s="48"/>
-      <c r="Q1" s="48"/>
-      <c r="R1" s="48"/>
-      <c r="S1" s="48"/>
-      <c r="T1" s="48"/>
-      <c r="U1" s="48"/>
-      <c r="V1" s="48"/>
-      <c r="W1" s="48"/>
-      <c r="X1" s="48"/>
-      <c r="Y1" s="48"/>
-      <c r="Z1" s="48"/>
-      <c r="AA1" s="48"/>
-      <c r="AB1" s="48"/>
-      <c r="AC1" s="48"/>
-      <c r="AD1" s="48"/>
-      <c r="AE1" s="48"/>
-      <c r="AF1" s="48"/>
-      <c r="AG1" s="48"/>
-      <c r="AH1" s="54"/>
-      <c r="AI1" s="55"/>
-      <c r="AJ1" s="55"/>
-      <c r="AK1" s="56" t="s">
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="40"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="40"/>
+      <c r="R1" s="40"/>
+      <c r="S1" s="40"/>
+      <c r="T1" s="40"/>
+      <c r="U1" s="40"/>
+      <c r="V1" s="40"/>
+      <c r="W1" s="40"/>
+      <c r="X1" s="40"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="40"/>
+      <c r="AA1" s="40"/>
+      <c r="AB1" s="40"/>
+      <c r="AC1" s="40"/>
+      <c r="AD1" s="40"/>
+      <c r="AE1" s="40"/>
+      <c r="AF1" s="40"/>
+      <c r="AG1" s="40"/>
+      <c r="AH1" s="40"/>
+      <c r="AI1" s="34"/>
+      <c r="AJ1" s="34"/>
+      <c r="AK1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="AL1" s="57"/>
-      <c r="AM1" s="57"/>
-      <c r="AN1" s="43"/>
-      <c r="AO1" s="44"/>
+      <c r="AL1" s="45"/>
+      <c r="AM1" s="45"/>
+      <c r="AN1" s="35"/>
+      <c r="AO1" s="36"/>
     </row>
     <row r="2" spans="1:43" ht="20" customHeight="1" thickBot="1">
       <c r="A2" s="4"/>
       <c r="B2" s="26"/>
       <c r="C2" s="26"/>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
-      <c r="H2" s="48"/>
-      <c r="I2" s="48"/>
-      <c r="J2" s="48"/>
-      <c r="K2" s="48"/>
-      <c r="L2" s="48"/>
-      <c r="M2" s="48"/>
-      <c r="N2" s="48"/>
-      <c r="O2" s="48"/>
-      <c r="P2" s="48"/>
-      <c r="Q2" s="48"/>
-      <c r="R2" s="48"/>
-      <c r="S2" s="48"/>
-      <c r="T2" s="48"/>
-      <c r="U2" s="48"/>
-      <c r="V2" s="48"/>
-      <c r="W2" s="48"/>
-      <c r="X2" s="48"/>
-      <c r="Y2" s="48"/>
-      <c r="Z2" s="48"/>
-      <c r="AA2" s="48"/>
-      <c r="AB2" s="48"/>
-      <c r="AC2" s="48"/>
-      <c r="AD2" s="48"/>
-      <c r="AE2" s="48"/>
-      <c r="AF2" s="48"/>
-      <c r="AG2" s="48"/>
-      <c r="AH2" s="54"/>
-      <c r="AI2" s="55"/>
-      <c r="AJ2" s="55"/>
-      <c r="AK2" s="56" t="s">
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="40"/>
+      <c r="O2" s="40"/>
+      <c r="P2" s="40"/>
+      <c r="Q2" s="40"/>
+      <c r="R2" s="40"/>
+      <c r="S2" s="40"/>
+      <c r="T2" s="40"/>
+      <c r="U2" s="40"/>
+      <c r="V2" s="40"/>
+      <c r="W2" s="40"/>
+      <c r="X2" s="40"/>
+      <c r="Y2" s="40"/>
+      <c r="Z2" s="40"/>
+      <c r="AA2" s="40"/>
+      <c r="AB2" s="40"/>
+      <c r="AC2" s="40"/>
+      <c r="AD2" s="40"/>
+      <c r="AE2" s="40"/>
+      <c r="AF2" s="40"/>
+      <c r="AG2" s="40"/>
+      <c r="AH2" s="40"/>
+      <c r="AI2" s="34"/>
+      <c r="AJ2" s="34"/>
+      <c r="AK2" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="AL2" s="57"/>
-      <c r="AM2" s="57"/>
-      <c r="AN2" s="45"/>
-      <c r="AO2" s="46"/>
+      <c r="AL2" s="45"/>
+      <c r="AM2" s="45"/>
+      <c r="AN2" s="37"/>
+      <c r="AO2" s="38"/>
     </row>
     <row r="3" spans="1:43">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="41" t="s">
+      <c r="B3" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="32" t="s">
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="32"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32" t="s">
+      <c r="F3" s="33"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="32"/>
-      <c r="J3" s="32"/>
-      <c r="K3" s="32" t="s">
+      <c r="I3" s="33"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="32"/>
-      <c r="M3" s="32"/>
-      <c r="N3" s="31" t="s">
+      <c r="L3" s="33"/>
+      <c r="M3" s="33"/>
+      <c r="N3" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="O3" s="32"/>
-      <c r="P3" s="32"/>
-      <c r="Q3" s="31" t="s">
+      <c r="O3" s="33"/>
+      <c r="P3" s="33"/>
+      <c r="Q3" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="R3" s="32"/>
-      <c r="S3" s="32"/>
-      <c r="T3" s="31" t="s">
+      <c r="R3" s="33"/>
+      <c r="S3" s="33"/>
+      <c r="T3" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="U3" s="32"/>
-      <c r="V3" s="32"/>
-      <c r="W3" s="31" t="s">
+      <c r="U3" s="33"/>
+      <c r="V3" s="33"/>
+      <c r="W3" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="X3" s="32"/>
-      <c r="Y3" s="32"/>
-      <c r="Z3" s="31" t="s">
+      <c r="X3" s="33"/>
+      <c r="Y3" s="33"/>
+      <c r="Z3" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="AA3" s="32"/>
-      <c r="AB3" s="32"/>
-      <c r="AC3" s="31" t="s">
+      <c r="AA3" s="33"/>
+      <c r="AB3" s="33"/>
+      <c r="AC3" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="AD3" s="32"/>
-      <c r="AE3" s="32"/>
-      <c r="AF3" s="31" t="s">
+      <c r="AD3" s="33"/>
+      <c r="AE3" s="33"/>
+      <c r="AF3" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="AG3" s="32"/>
-      <c r="AH3" s="32"/>
-      <c r="AI3" s="32" t="s">
+      <c r="AG3" s="33"/>
+      <c r="AH3" s="33"/>
+      <c r="AI3" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="AJ3" s="32"/>
-      <c r="AK3" s="32"/>
-      <c r="AL3" s="52" t="s">
+      <c r="AJ3" s="33"/>
+      <c r="AK3" s="33"/>
+      <c r="AL3" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="AM3" s="49"/>
-      <c r="AN3" s="50"/>
-      <c r="AO3" s="35" t="s">
+      <c r="AM3" s="42"/>
+      <c r="AN3" s="43"/>
+      <c r="AO3" s="53" t="s">
         <v>9</v>
       </c>
       <c r="AP3" s="19"/>
       <c r="AQ3" s="19"/>
     </row>
     <row r="4" spans="1:43">
-      <c r="A4" s="40"/>
+      <c r="A4" s="47"/>
       <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
@@ -1378,16 +1378,16 @@
       <c r="AK4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="AL4" s="51" t="s">
+      <c r="AL4" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="AM4" s="51" t="s">
+      <c r="AM4" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="AN4" s="53" t="s">
+      <c r="AN4" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="AO4" s="35"/>
+      <c r="AO4" s="53"/>
       <c r="AP4" s="20"/>
       <c r="AQ4" s="21"/>
     </row>
@@ -1483,7 +1483,7 @@
       <c r="AL6" s="12"/>
       <c r="AM6" s="12"/>
       <c r="AN6" s="12"/>
-      <c r="AO6" s="36"/>
+      <c r="AO6" s="54"/>
       <c r="AP6" s="22"/>
       <c r="AQ6" s="22"/>
     </row>
@@ -1530,7 +1530,7 @@
       <c r="AL7" s="12"/>
       <c r="AM7" s="12"/>
       <c r="AN7" s="13"/>
-      <c r="AO7" s="37"/>
+      <c r="AO7" s="55"/>
       <c r="AP7" s="22"/>
       <c r="AQ7" s="22"/>
     </row>
@@ -1577,7 +1577,7 @@
       <c r="AL8" s="12"/>
       <c r="AM8" s="12"/>
       <c r="AN8" s="13"/>
-      <c r="AO8" s="37"/>
+      <c r="AO8" s="55"/>
       <c r="AP8" s="22"/>
       <c r="AQ8" s="22"/>
     </row>
@@ -1624,7 +1624,7 @@
       <c r="AL9" s="12"/>
       <c r="AM9" s="12"/>
       <c r="AN9" s="13"/>
-      <c r="AO9" s="37"/>
+      <c r="AO9" s="55"/>
       <c r="AP9" s="22"/>
       <c r="AQ9" s="22"/>
     </row>
@@ -1671,7 +1671,7 @@
       <c r="AL10" s="12"/>
       <c r="AM10" s="12"/>
       <c r="AN10" s="13"/>
-      <c r="AO10" s="37"/>
+      <c r="AO10" s="55"/>
       <c r="AP10" s="22"/>
       <c r="AQ10" s="22"/>
     </row>
@@ -1718,7 +1718,7 @@
       <c r="AL11" s="12"/>
       <c r="AM11" s="12"/>
       <c r="AN11" s="13"/>
-      <c r="AO11" s="37"/>
+      <c r="AO11" s="55"/>
       <c r="AP11" s="22"/>
       <c r="AQ11" s="22"/>
     </row>
@@ -1765,7 +1765,7 @@
       <c r="AL12" s="12"/>
       <c r="AM12" s="12"/>
       <c r="AN12" s="12"/>
-      <c r="AO12" s="37"/>
+      <c r="AO12" s="55"/>
       <c r="AP12" s="22"/>
       <c r="AQ12" s="22"/>
     </row>
@@ -1812,7 +1812,7 @@
       <c r="AL13" s="12"/>
       <c r="AM13" s="12"/>
       <c r="AN13" s="12"/>
-      <c r="AO13" s="38"/>
+      <c r="AO13" s="56"/>
       <c r="AP13" s="22"/>
       <c r="AQ13" s="22"/>
     </row>
@@ -2004,7 +2004,7 @@
       <c r="AL17" s="11"/>
       <c r="AM17" s="11"/>
       <c r="AN17" s="13"/>
-      <c r="AO17" s="36"/>
+      <c r="AO17" s="54"/>
       <c r="AP17" s="23"/>
       <c r="AQ17" s="23"/>
     </row>
@@ -2051,7 +2051,7 @@
       <c r="AL18" s="11"/>
       <c r="AM18" s="11"/>
       <c r="AN18" s="13"/>
-      <c r="AO18" s="37"/>
+      <c r="AO18" s="55"/>
       <c r="AP18" s="23"/>
       <c r="AQ18" s="23"/>
     </row>
@@ -2098,7 +2098,7 @@
       <c r="AL19" s="12"/>
       <c r="AM19" s="12"/>
       <c r="AN19" s="12"/>
-      <c r="AO19" s="37"/>
+      <c r="AO19" s="55"/>
       <c r="AP19" s="22"/>
       <c r="AQ19" s="22"/>
     </row>
@@ -2145,7 +2145,7 @@
       <c r="AL20" s="12"/>
       <c r="AM20" s="12"/>
       <c r="AN20" s="12"/>
-      <c r="AO20" s="37"/>
+      <c r="AO20" s="55"/>
       <c r="AP20" s="22"/>
       <c r="AQ20" s="22"/>
     </row>
@@ -2192,7 +2192,7 @@
       <c r="AL21" s="12"/>
       <c r="AM21" s="12"/>
       <c r="AN21" s="13"/>
-      <c r="AO21" s="37"/>
+      <c r="AO21" s="55"/>
       <c r="AP21" s="22"/>
       <c r="AQ21" s="22"/>
     </row>
@@ -2239,7 +2239,7 @@
       <c r="AL22" s="12"/>
       <c r="AM22" s="12"/>
       <c r="AN22" s="13"/>
-      <c r="AO22" s="37"/>
+      <c r="AO22" s="55"/>
       <c r="AP22" s="22"/>
       <c r="AQ22" s="22"/>
     </row>
@@ -2286,7 +2286,7 @@
       <c r="AL23" s="12"/>
       <c r="AM23" s="12"/>
       <c r="AN23" s="13"/>
-      <c r="AO23" s="37"/>
+      <c r="AO23" s="55"/>
       <c r="AP23" s="22"/>
       <c r="AQ23" s="22"/>
     </row>
@@ -2333,7 +2333,7 @@
       <c r="AL24" s="12"/>
       <c r="AM24" s="12"/>
       <c r="AN24" s="13"/>
-      <c r="AO24" s="38"/>
+      <c r="AO24" s="56"/>
       <c r="AP24" s="22"/>
       <c r="AQ24" s="22"/>
     </row>
@@ -2525,7 +2525,7 @@
       <c r="AL28" s="12"/>
       <c r="AM28" s="12"/>
       <c r="AN28" s="13"/>
-      <c r="AO28" s="36"/>
+      <c r="AO28" s="54"/>
       <c r="AP28" s="22"/>
       <c r="AQ28" s="22"/>
     </row>
@@ -2572,7 +2572,7 @@
       <c r="AL29" s="12"/>
       <c r="AM29" s="12"/>
       <c r="AN29" s="13"/>
-      <c r="AO29" s="37"/>
+      <c r="AO29" s="55"/>
       <c r="AP29" s="22"/>
       <c r="AQ29" s="22"/>
     </row>
@@ -2619,7 +2619,7 @@
       <c r="AL30" s="12"/>
       <c r="AM30" s="12"/>
       <c r="AN30" s="13"/>
-      <c r="AO30" s="37"/>
+      <c r="AO30" s="55"/>
       <c r="AP30" s="22"/>
       <c r="AQ30" s="22"/>
     </row>
@@ -2666,7 +2666,7 @@
       <c r="AL31" s="12"/>
       <c r="AM31" s="12"/>
       <c r="AN31" s="13"/>
-      <c r="AO31" s="37"/>
+      <c r="AO31" s="55"/>
       <c r="AP31" s="22"/>
       <c r="AQ31" s="22"/>
     </row>
@@ -2713,7 +2713,7 @@
       <c r="AL32" s="12"/>
       <c r="AM32" s="12"/>
       <c r="AN32" s="13"/>
-      <c r="AO32" s="37"/>
+      <c r="AO32" s="55"/>
       <c r="AP32" s="22"/>
       <c r="AQ32" s="22"/>
     </row>
@@ -2760,7 +2760,7 @@
       <c r="AL33" s="12"/>
       <c r="AM33" s="12"/>
       <c r="AN33" s="12"/>
-      <c r="AO33" s="37"/>
+      <c r="AO33" s="55"/>
       <c r="AP33" s="22"/>
       <c r="AQ33" s="22"/>
     </row>
@@ -2807,7 +2807,7 @@
       <c r="AL34" s="12"/>
       <c r="AM34" s="12"/>
       <c r="AN34" s="12"/>
-      <c r="AO34" s="38"/>
+      <c r="AO34" s="56"/>
       <c r="AP34" s="22"/>
       <c r="AQ34" s="22"/>
     </row>
@@ -2862,71 +2862,110 @@
     </row>
     <row r="36" spans="1:43" ht="15" thickBot="1">
       <c r="A36" s="14"/>
-      <c r="B36" s="30" t="s">
+      <c r="B36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="30"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="30" t="s">
+      <c r="C36" s="50"/>
+      <c r="D36" s="16">
+        <f>SUM(D5:D35)</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="F36" s="30"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="30" t="s">
+      <c r="F36" s="50"/>
+      <c r="G36" s="59">
+        <f>SUM(G5:G35)</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="I36" s="30"/>
-      <c r="J36" s="16"/>
-      <c r="K36" s="30" t="s">
+      <c r="I36" s="50"/>
+      <c r="J36" s="59">
+        <f>SUM(J5:J35)</f>
+        <v>0</v>
+      </c>
+      <c r="K36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="L36" s="30"/>
-      <c r="M36" s="15"/>
-      <c r="N36" s="30" t="s">
+      <c r="L36" s="50"/>
+      <c r="M36" s="15">
+        <f>SUM(M5:M35)</f>
+        <v>0</v>
+      </c>
+      <c r="N36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="O36" s="30"/>
-      <c r="P36" s="15"/>
-      <c r="Q36" s="30" t="s">
+      <c r="O36" s="50"/>
+      <c r="P36" s="15">
+        <f>SUM(P5:P35)</f>
+        <v>0</v>
+      </c>
+      <c r="Q36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="R36" s="30"/>
-      <c r="S36" s="15"/>
-      <c r="T36" s="30" t="s">
+      <c r="R36" s="50"/>
+      <c r="S36" s="15">
+        <f>SUM(S5:S35)</f>
+        <v>0</v>
+      </c>
+      <c r="T36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="U36" s="30"/>
-      <c r="V36" s="15"/>
-      <c r="W36" s="30" t="s">
+      <c r="U36" s="50"/>
+      <c r="V36" s="15">
+        <f>SUM(V5:V35)</f>
+        <v>0</v>
+      </c>
+      <c r="W36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="X36" s="30"/>
-      <c r="Y36" s="15"/>
-      <c r="Z36" s="30" t="s">
+      <c r="X36" s="50"/>
+      <c r="Y36" s="15">
+        <f>SUM(Y5:Y35)</f>
+        <v>0</v>
+      </c>
+      <c r="Z36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="AA36" s="30"/>
-      <c r="AB36" s="15"/>
-      <c r="AC36" s="30" t="s">
+      <c r="AA36" s="50"/>
+      <c r="AB36" s="15">
+        <f>SUM(AB5:AB35)</f>
+        <v>0</v>
+      </c>
+      <c r="AC36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="AD36" s="30"/>
-      <c r="AE36" s="15"/>
-      <c r="AF36" s="30" t="s">
+      <c r="AD36" s="50"/>
+      <c r="AE36" s="15">
+        <f>SUM(AE5:AE35)</f>
+        <v>0</v>
+      </c>
+      <c r="AF36" s="50" t="s">
         <v>18</v>
       </c>
-      <c r="AG36" s="30"/>
-      <c r="AH36" s="15"/>
-      <c r="AI36" s="33" t="s">
+      <c r="AG36" s="50"/>
+      <c r="AH36" s="15">
+        <f>SUM(AH5:AH35)</f>
+        <v>0</v>
+      </c>
+      <c r="AI36" s="51" t="s">
         <v>18</v>
       </c>
-      <c r="AJ36" s="33"/>
-      <c r="AK36" s="29"/>
-      <c r="AL36" s="59" t="s">
+      <c r="AJ36" s="51"/>
+      <c r="AK36" s="29">
+        <f>SUM(AK5:AK35)</f>
+        <v>0</v>
+      </c>
+      <c r="AL36" s="57" t="s">
         <v>18</v>
       </c>
       <c r="AM36" s="58"/>
-      <c r="AN36" s="10"/>
+      <c r="AN36" s="10">
+        <f>SUM(AN5:AN35)</f>
+        <v>0</v>
+      </c>
       <c r="AO36" s="28"/>
       <c r="AP36" s="24"/>
       <c r="AQ36" s="24"/>
@@ -2939,18 +2978,46 @@
       <c r="O37" s="17"/>
       <c r="P37" s="17"/>
       <c r="T37" s="3"/>
-      <c r="AI37" s="34" t="s">
+      <c r="AI37" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="AJ37" s="34"/>
-      <c r="AK37" s="34"/>
-      <c r="AL37" s="34"/>
-      <c r="AM37" s="34"/>
-      <c r="AN37" s="34"/>
-      <c r="AO37" s="34"/>
+      <c r="AJ37" s="52"/>
+      <c r="AK37" s="52"/>
+      <c r="AL37" s="52"/>
+      <c r="AM37" s="52"/>
+      <c r="AN37" s="52"/>
+      <c r="AO37" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="40">
+    <mergeCell ref="AI36:AJ36"/>
+    <mergeCell ref="AI37:AO37"/>
+    <mergeCell ref="AO3:AO4"/>
+    <mergeCell ref="AO6:AO13"/>
+    <mergeCell ref="AO17:AO24"/>
+    <mergeCell ref="AO28:AO34"/>
+    <mergeCell ref="AL36:AM36"/>
+    <mergeCell ref="Q36:R36"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="T36:U36"/>
+    <mergeCell ref="AF3:AH3"/>
+    <mergeCell ref="AF36:AG36"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="W36:X36"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z36:AA36"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC36:AD36"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="AI1:AJ1"/>
     <mergeCell ref="AN1:AO1"/>
@@ -2962,35 +3029,7 @@
     <mergeCell ref="AL3:AN3"/>
     <mergeCell ref="AK1:AM1"/>
     <mergeCell ref="AK2:AM2"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="N36:O36"/>
     <mergeCell ref="Q3:S3"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="T36:U36"/>
-    <mergeCell ref="AF3:AH3"/>
-    <mergeCell ref="AF36:AG36"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="W36:X36"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z36:AA36"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC36:AD36"/>
-    <mergeCell ref="AI36:AJ36"/>
-    <mergeCell ref="AI37:AO37"/>
-    <mergeCell ref="AO3:AO4"/>
-    <mergeCell ref="AO6:AO13"/>
-    <mergeCell ref="AO17:AO24"/>
-    <mergeCell ref="AO28:AO34"/>
-    <mergeCell ref="AL36:AM36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat: add custom validation messages for alat kalibrasi form
</commit_message>
<xml_diff>
--- a/public/assets/templates/utility/laporan_air_utility.xlsx
+++ b/public/assets/templates/utility/laporan_air_utility.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\utility\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C403ED4F-C85D-4293-ADB8-3DCECD69851C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1108955E-7FE8-4305-9846-31D1B8E8469A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{99CC749A-043A-42C9-9CA5-3CA614D07719}"/>
   </bookViews>
@@ -540,9 +540,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -588,12 +585,54 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -630,46 +669,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1092,7 +1092,7 @@
     <col min="16" max="16" width="8.54296875" style="3" customWidth="1"/>
     <col min="17" max="18" width="7.1796875" style="3" customWidth="1"/>
     <col min="19" max="19" width="8.26953125" style="3" customWidth="1"/>
-    <col min="20" max="20" width="8" style="18" customWidth="1"/>
+    <col min="20" max="20" width="8" style="17" customWidth="1"/>
     <col min="21" max="39" width="9.1796875" style="3"/>
     <col min="40" max="40" width="8.7265625" style="3" customWidth="1"/>
     <col min="41" max="41" width="18.7265625" style="3" customWidth="1"/>
@@ -1103,173 +1103,173 @@
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
-      <c r="D1" s="39" t="s">
+      <c r="D1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
-      <c r="M1" s="40"/>
-      <c r="N1" s="40"/>
-      <c r="O1" s="40"/>
-      <c r="P1" s="40"/>
-      <c r="Q1" s="40"/>
-      <c r="R1" s="40"/>
-      <c r="S1" s="40"/>
-      <c r="T1" s="40"/>
-      <c r="U1" s="40"/>
-      <c r="V1" s="40"/>
-      <c r="W1" s="40"/>
-      <c r="X1" s="40"/>
-      <c r="Y1" s="40"/>
-      <c r="Z1" s="40"/>
-      <c r="AA1" s="40"/>
-      <c r="AB1" s="40"/>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-      <c r="AF1" s="40"/>
-      <c r="AG1" s="40"/>
-      <c r="AH1" s="40"/>
-      <c r="AI1" s="34"/>
-      <c r="AJ1" s="34"/>
-      <c r="AK1" s="44" t="s">
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="53"/>
+      <c r="P1" s="53"/>
+      <c r="Q1" s="53"/>
+      <c r="R1" s="53"/>
+      <c r="S1" s="53"/>
+      <c r="T1" s="53"/>
+      <c r="U1" s="53"/>
+      <c r="V1" s="53"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="53"/>
+      <c r="Y1" s="53"/>
+      <c r="Z1" s="53"/>
+      <c r="AA1" s="53"/>
+      <c r="AB1" s="53"/>
+      <c r="AC1" s="53"/>
+      <c r="AD1" s="53"/>
+      <c r="AE1" s="53"/>
+      <c r="AF1" s="53"/>
+      <c r="AG1" s="53"/>
+      <c r="AH1" s="53"/>
+      <c r="AI1" s="47"/>
+      <c r="AJ1" s="47"/>
+      <c r="AK1" s="57" t="s">
         <v>1</v>
       </c>
-      <c r="AL1" s="45"/>
-      <c r="AM1" s="45"/>
-      <c r="AN1" s="35"/>
-      <c r="AO1" s="36"/>
+      <c r="AL1" s="58"/>
+      <c r="AM1" s="58"/>
+      <c r="AN1" s="48"/>
+      <c r="AO1" s="49"/>
     </row>
     <row r="2" spans="1:43" ht="20" customHeight="1" thickBot="1">
       <c r="A2" s="4"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="39" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="40"/>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="40"/>
-      <c r="S2" s="40"/>
-      <c r="T2" s="40"/>
-      <c r="U2" s="40"/>
-      <c r="V2" s="40"/>
-      <c r="W2" s="40"/>
-      <c r="X2" s="40"/>
-      <c r="Y2" s="40"/>
-      <c r="Z2" s="40"/>
-      <c r="AA2" s="40"/>
-      <c r="AB2" s="40"/>
-      <c r="AC2" s="40"/>
-      <c r="AD2" s="40"/>
-      <c r="AE2" s="40"/>
-      <c r="AF2" s="40"/>
-      <c r="AG2" s="40"/>
-      <c r="AH2" s="40"/>
-      <c r="AI2" s="34"/>
-      <c r="AJ2" s="34"/>
-      <c r="AK2" s="44" t="s">
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
+      <c r="M2" s="53"/>
+      <c r="N2" s="53"/>
+      <c r="O2" s="53"/>
+      <c r="P2" s="53"/>
+      <c r="Q2" s="53"/>
+      <c r="R2" s="53"/>
+      <c r="S2" s="53"/>
+      <c r="T2" s="53"/>
+      <c r="U2" s="53"/>
+      <c r="V2" s="53"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="53"/>
+      <c r="Y2" s="53"/>
+      <c r="Z2" s="53"/>
+      <c r="AA2" s="53"/>
+      <c r="AB2" s="53"/>
+      <c r="AC2" s="53"/>
+      <c r="AD2" s="53"/>
+      <c r="AE2" s="53"/>
+      <c r="AF2" s="53"/>
+      <c r="AG2" s="53"/>
+      <c r="AH2" s="53"/>
+      <c r="AI2" s="47"/>
+      <c r="AJ2" s="47"/>
+      <c r="AK2" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="AL2" s="45"/>
-      <c r="AM2" s="45"/>
-      <c r="AN2" s="37"/>
-      <c r="AO2" s="38"/>
+      <c r="AL2" s="58"/>
+      <c r="AM2" s="58"/>
+      <c r="AN2" s="50"/>
+      <c r="AO2" s="51"/>
     </row>
     <row r="3" spans="1:43">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="48" t="s">
+      <c r="B3" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="33" t="s">
+      <c r="C3" s="46"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="33"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="33" t="s">
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
+      <c r="H3" s="42" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="33"/>
-      <c r="J3" s="33"/>
-      <c r="K3" s="33" t="s">
+      <c r="I3" s="42"/>
+      <c r="J3" s="42"/>
+      <c r="K3" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="32" t="s">
+      <c r="L3" s="42"/>
+      <c r="M3" s="42"/>
+      <c r="N3" s="41" t="s">
         <v>22</v>
       </c>
-      <c r="O3" s="33"/>
-      <c r="P3" s="33"/>
-      <c r="Q3" s="32" t="s">
+      <c r="O3" s="42"/>
+      <c r="P3" s="42"/>
+      <c r="Q3" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="R3" s="33"/>
-      <c r="S3" s="33"/>
-      <c r="T3" s="32" t="s">
+      <c r="R3" s="42"/>
+      <c r="S3" s="42"/>
+      <c r="T3" s="41" t="s">
         <v>24</v>
       </c>
-      <c r="U3" s="33"/>
-      <c r="V3" s="33"/>
-      <c r="W3" s="32" t="s">
+      <c r="U3" s="42"/>
+      <c r="V3" s="42"/>
+      <c r="W3" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="X3" s="33"/>
-      <c r="Y3" s="33"/>
-      <c r="Z3" s="32" t="s">
+      <c r="X3" s="42"/>
+      <c r="Y3" s="42"/>
+      <c r="Z3" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="AA3" s="33"/>
-      <c r="AB3" s="33"/>
-      <c r="AC3" s="32" t="s">
+      <c r="AA3" s="42"/>
+      <c r="AB3" s="42"/>
+      <c r="AC3" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="AD3" s="33"/>
-      <c r="AE3" s="33"/>
-      <c r="AF3" s="32" t="s">
+      <c r="AD3" s="42"/>
+      <c r="AE3" s="42"/>
+      <c r="AF3" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="AG3" s="33"/>
-      <c r="AH3" s="33"/>
-      <c r="AI3" s="33" t="s">
+      <c r="AG3" s="42"/>
+      <c r="AH3" s="42"/>
+      <c r="AI3" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="AJ3" s="33"/>
-      <c r="AK3" s="33"/>
-      <c r="AL3" s="41" t="s">
+      <c r="AJ3" s="42"/>
+      <c r="AK3" s="42"/>
+      <c r="AL3" s="54" t="s">
         <v>29</v>
       </c>
-      <c r="AM3" s="42"/>
-      <c r="AN3" s="43"/>
-      <c r="AO3" s="53" t="s">
+      <c r="AM3" s="55"/>
+      <c r="AN3" s="56"/>
+      <c r="AO3" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="AP3" s="19"/>
-      <c r="AQ3" s="19"/>
+      <c r="AP3" s="18"/>
+      <c r="AQ3" s="18"/>
     </row>
     <row r="4" spans="1:43">
-      <c r="A4" s="47"/>
+      <c r="A4" s="44"/>
       <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
@@ -1378,18 +1378,18 @@
       <c r="AK4" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="AL4" s="30" t="s">
+      <c r="AL4" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="AM4" s="30" t="s">
+      <c r="AM4" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="AN4" s="31" t="s">
+      <c r="AN4" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="AO4" s="53"/>
-      <c r="AP4" s="20"/>
-      <c r="AQ4" s="21"/>
+      <c r="AO4" s="34"/>
+      <c r="AP4" s="19"/>
+      <c r="AQ4" s="20"/>
     </row>
     <row r="5" spans="1:43" ht="17" customHeight="1">
       <c r="A5" s="9">
@@ -1434,11 +1434,11 @@
       <c r="AL5" s="12"/>
       <c r="AM5" s="12"/>
       <c r="AN5" s="12"/>
-      <c r="AO5" s="25" t="s">
+      <c r="AO5" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="AP5" s="22"/>
-      <c r="AQ5" s="22"/>
+      <c r="AP5" s="21"/>
+      <c r="AQ5" s="21"/>
     </row>
     <row r="6" spans="1:43" ht="17" customHeight="1">
       <c r="A6" s="9">
@@ -1483,9 +1483,9 @@
       <c r="AL6" s="12"/>
       <c r="AM6" s="12"/>
       <c r="AN6" s="12"/>
-      <c r="AO6" s="54"/>
-      <c r="AP6" s="22"/>
-      <c r="AQ6" s="22"/>
+      <c r="AO6" s="35"/>
+      <c r="AP6" s="21"/>
+      <c r="AQ6" s="21"/>
     </row>
     <row r="7" spans="1:43" ht="17" customHeight="1">
       <c r="A7" s="9">
@@ -1530,9 +1530,9 @@
       <c r="AL7" s="12"/>
       <c r="AM7" s="12"/>
       <c r="AN7" s="13"/>
-      <c r="AO7" s="55"/>
-      <c r="AP7" s="22"/>
-      <c r="AQ7" s="22"/>
+      <c r="AO7" s="36"/>
+      <c r="AP7" s="21"/>
+      <c r="AQ7" s="21"/>
     </row>
     <row r="8" spans="1:43" ht="17" customHeight="1">
       <c r="A8" s="9">
@@ -1577,9 +1577,9 @@
       <c r="AL8" s="12"/>
       <c r="AM8" s="12"/>
       <c r="AN8" s="13"/>
-      <c r="AO8" s="55"/>
-      <c r="AP8" s="22"/>
-      <c r="AQ8" s="22"/>
+      <c r="AO8" s="36"/>
+      <c r="AP8" s="21"/>
+      <c r="AQ8" s="21"/>
     </row>
     <row r="9" spans="1:43" ht="17" customHeight="1">
       <c r="A9" s="9">
@@ -1624,9 +1624,9 @@
       <c r="AL9" s="12"/>
       <c r="AM9" s="12"/>
       <c r="AN9" s="13"/>
-      <c r="AO9" s="55"/>
-      <c r="AP9" s="22"/>
-      <c r="AQ9" s="22"/>
+      <c r="AO9" s="36"/>
+      <c r="AP9" s="21"/>
+      <c r="AQ9" s="21"/>
     </row>
     <row r="10" spans="1:43" ht="17" customHeight="1">
       <c r="A10" s="9">
@@ -1671,9 +1671,9 @@
       <c r="AL10" s="12"/>
       <c r="AM10" s="12"/>
       <c r="AN10" s="13"/>
-      <c r="AO10" s="55"/>
-      <c r="AP10" s="22"/>
-      <c r="AQ10" s="22"/>
+      <c r="AO10" s="36"/>
+      <c r="AP10" s="21"/>
+      <c r="AQ10" s="21"/>
     </row>
     <row r="11" spans="1:43" ht="17" customHeight="1">
       <c r="A11" s="9">
@@ -1718,9 +1718,9 @@
       <c r="AL11" s="12"/>
       <c r="AM11" s="12"/>
       <c r="AN11" s="13"/>
-      <c r="AO11" s="55"/>
-      <c r="AP11" s="22"/>
-      <c r="AQ11" s="22"/>
+      <c r="AO11" s="36"/>
+      <c r="AP11" s="21"/>
+      <c r="AQ11" s="21"/>
     </row>
     <row r="12" spans="1:43" ht="17" customHeight="1">
       <c r="A12" s="9">
@@ -1765,9 +1765,9 @@
       <c r="AL12" s="12"/>
       <c r="AM12" s="12"/>
       <c r="AN12" s="12"/>
-      <c r="AO12" s="55"/>
-      <c r="AP12" s="22"/>
-      <c r="AQ12" s="22"/>
+      <c r="AO12" s="36"/>
+      <c r="AP12" s="21"/>
+      <c r="AQ12" s="21"/>
     </row>
     <row r="13" spans="1:43" ht="17" customHeight="1">
       <c r="A13" s="9">
@@ -1812,9 +1812,9 @@
       <c r="AL13" s="12"/>
       <c r="AM13" s="12"/>
       <c r="AN13" s="12"/>
-      <c r="AO13" s="56"/>
-      <c r="AP13" s="22"/>
-      <c r="AQ13" s="22"/>
+      <c r="AO13" s="37"/>
+      <c r="AP13" s="21"/>
+      <c r="AQ13" s="21"/>
     </row>
     <row r="14" spans="1:43" ht="17" customHeight="1">
       <c r="A14" s="9">
@@ -1859,11 +1859,11 @@
       <c r="AL14" s="11"/>
       <c r="AM14" s="11"/>
       <c r="AN14" s="13"/>
-      <c r="AO14" s="27" t="s">
+      <c r="AO14" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="AP14" s="23"/>
-      <c r="AQ14" s="23"/>
+      <c r="AP14" s="22"/>
+      <c r="AQ14" s="22"/>
     </row>
     <row r="15" spans="1:43" ht="17" customHeight="1">
       <c r="A15" s="9">
@@ -1908,9 +1908,9 @@
       <c r="AL15" s="11"/>
       <c r="AM15" s="11"/>
       <c r="AN15" s="13"/>
-      <c r="AO15" s="28"/>
-      <c r="AP15" s="23"/>
-      <c r="AQ15" s="23"/>
+      <c r="AO15" s="27"/>
+      <c r="AP15" s="22"/>
+      <c r="AQ15" s="22"/>
     </row>
     <row r="16" spans="1:43" ht="17" customHeight="1">
       <c r="A16" s="9">
@@ -1955,11 +1955,11 @@
       <c r="AL16" s="11"/>
       <c r="AM16" s="11"/>
       <c r="AN16" s="13"/>
-      <c r="AO16" s="25" t="s">
+      <c r="AO16" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="AP16" s="23"/>
-      <c r="AQ16" s="23"/>
+      <c r="AP16" s="22"/>
+      <c r="AQ16" s="22"/>
     </row>
     <row r="17" spans="1:43" ht="17" customHeight="1">
       <c r="A17" s="9">
@@ -2004,9 +2004,9 @@
       <c r="AL17" s="11"/>
       <c r="AM17" s="11"/>
       <c r="AN17" s="13"/>
-      <c r="AO17" s="54"/>
-      <c r="AP17" s="23"/>
-      <c r="AQ17" s="23"/>
+      <c r="AO17" s="35"/>
+      <c r="AP17" s="22"/>
+      <c r="AQ17" s="22"/>
     </row>
     <row r="18" spans="1:43" ht="17" customHeight="1">
       <c r="A18" s="9">
@@ -2051,9 +2051,9 @@
       <c r="AL18" s="11"/>
       <c r="AM18" s="11"/>
       <c r="AN18" s="13"/>
-      <c r="AO18" s="55"/>
-      <c r="AP18" s="23"/>
-      <c r="AQ18" s="23"/>
+      <c r="AO18" s="36"/>
+      <c r="AP18" s="22"/>
+      <c r="AQ18" s="22"/>
     </row>
     <row r="19" spans="1:43" ht="17" customHeight="1">
       <c r="A19" s="9">
@@ -2098,9 +2098,9 @@
       <c r="AL19" s="12"/>
       <c r="AM19" s="12"/>
       <c r="AN19" s="12"/>
-      <c r="AO19" s="55"/>
-      <c r="AP19" s="22"/>
-      <c r="AQ19" s="22"/>
+      <c r="AO19" s="36"/>
+      <c r="AP19" s="21"/>
+      <c r="AQ19" s="21"/>
     </row>
     <row r="20" spans="1:43" ht="17" customHeight="1">
       <c r="A20" s="9">
@@ -2145,9 +2145,9 @@
       <c r="AL20" s="12"/>
       <c r="AM20" s="12"/>
       <c r="AN20" s="12"/>
-      <c r="AO20" s="55"/>
-      <c r="AP20" s="22"/>
-      <c r="AQ20" s="22"/>
+      <c r="AO20" s="36"/>
+      <c r="AP20" s="21"/>
+      <c r="AQ20" s="21"/>
     </row>
     <row r="21" spans="1:43" ht="17" customHeight="1">
       <c r="A21" s="9">
@@ -2192,9 +2192,9 @@
       <c r="AL21" s="12"/>
       <c r="AM21" s="12"/>
       <c r="AN21" s="13"/>
-      <c r="AO21" s="55"/>
-      <c r="AP21" s="22"/>
-      <c r="AQ21" s="22"/>
+      <c r="AO21" s="36"/>
+      <c r="AP21" s="21"/>
+      <c r="AQ21" s="21"/>
     </row>
     <row r="22" spans="1:43" ht="17" customHeight="1">
       <c r="A22" s="9">
@@ -2239,9 +2239,9 @@
       <c r="AL22" s="12"/>
       <c r="AM22" s="12"/>
       <c r="AN22" s="13"/>
-      <c r="AO22" s="55"/>
-      <c r="AP22" s="22"/>
-      <c r="AQ22" s="22"/>
+      <c r="AO22" s="36"/>
+      <c r="AP22" s="21"/>
+      <c r="AQ22" s="21"/>
     </row>
     <row r="23" spans="1:43" ht="17" customHeight="1">
       <c r="A23" s="9">
@@ -2286,9 +2286,9 @@
       <c r="AL23" s="12"/>
       <c r="AM23" s="12"/>
       <c r="AN23" s="13"/>
-      <c r="AO23" s="55"/>
-      <c r="AP23" s="22"/>
-      <c r="AQ23" s="22"/>
+      <c r="AO23" s="36"/>
+      <c r="AP23" s="21"/>
+      <c r="AQ23" s="21"/>
     </row>
     <row r="24" spans="1:43" ht="17" customHeight="1">
       <c r="A24" s="9">
@@ -2333,9 +2333,9 @@
       <c r="AL24" s="12"/>
       <c r="AM24" s="12"/>
       <c r="AN24" s="13"/>
-      <c r="AO24" s="56"/>
-      <c r="AP24" s="22"/>
-      <c r="AQ24" s="22"/>
+      <c r="AO24" s="37"/>
+      <c r="AP24" s="21"/>
+      <c r="AQ24" s="21"/>
     </row>
     <row r="25" spans="1:43" ht="17" customHeight="1">
       <c r="A25" s="9">
@@ -2380,11 +2380,11 @@
       <c r="AL25" s="12"/>
       <c r="AM25" s="12"/>
       <c r="AN25" s="13"/>
-      <c r="AO25" s="27" t="s">
+      <c r="AO25" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="AP25" s="22"/>
-      <c r="AQ25" s="22"/>
+      <c r="AP25" s="21"/>
+      <c r="AQ25" s="21"/>
     </row>
     <row r="26" spans="1:43" ht="17" customHeight="1">
       <c r="A26" s="9">
@@ -2429,9 +2429,9 @@
       <c r="AL26" s="12"/>
       <c r="AM26" s="12"/>
       <c r="AN26" s="12"/>
-      <c r="AO26" s="28"/>
-      <c r="AP26" s="22"/>
-      <c r="AQ26" s="22"/>
+      <c r="AO26" s="27"/>
+      <c r="AP26" s="21"/>
+      <c r="AQ26" s="21"/>
     </row>
     <row r="27" spans="1:43" ht="17" customHeight="1">
       <c r="A27" s="9">
@@ -2476,11 +2476,11 @@
       <c r="AL27" s="12"/>
       <c r="AM27" s="12"/>
       <c r="AN27" s="12"/>
-      <c r="AO27" s="25" t="s">
+      <c r="AO27" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="AP27" s="22"/>
-      <c r="AQ27" s="22"/>
+      <c r="AP27" s="21"/>
+      <c r="AQ27" s="21"/>
     </row>
     <row r="28" spans="1:43" ht="17" customHeight="1">
       <c r="A28" s="9">
@@ -2525,9 +2525,9 @@
       <c r="AL28" s="12"/>
       <c r="AM28" s="12"/>
       <c r="AN28" s="13"/>
-      <c r="AO28" s="54"/>
-      <c r="AP28" s="22"/>
-      <c r="AQ28" s="22"/>
+      <c r="AO28" s="35"/>
+      <c r="AP28" s="21"/>
+      <c r="AQ28" s="21"/>
     </row>
     <row r="29" spans="1:43" ht="17" customHeight="1">
       <c r="A29" s="9">
@@ -2572,9 +2572,9 @@
       <c r="AL29" s="12"/>
       <c r="AM29" s="12"/>
       <c r="AN29" s="13"/>
-      <c r="AO29" s="55"/>
-      <c r="AP29" s="22"/>
-      <c r="AQ29" s="22"/>
+      <c r="AO29" s="36"/>
+      <c r="AP29" s="21"/>
+      <c r="AQ29" s="21"/>
     </row>
     <row r="30" spans="1:43" ht="17" customHeight="1">
       <c r="A30" s="9">
@@ -2619,9 +2619,9 @@
       <c r="AL30" s="12"/>
       <c r="AM30" s="12"/>
       <c r="AN30" s="13"/>
-      <c r="AO30" s="55"/>
-      <c r="AP30" s="22"/>
-      <c r="AQ30" s="22"/>
+      <c r="AO30" s="36"/>
+      <c r="AP30" s="21"/>
+      <c r="AQ30" s="21"/>
     </row>
     <row r="31" spans="1:43" ht="17" customHeight="1">
       <c r="A31" s="9">
@@ -2666,9 +2666,9 @@
       <c r="AL31" s="12"/>
       <c r="AM31" s="12"/>
       <c r="AN31" s="13"/>
-      <c r="AO31" s="55"/>
-      <c r="AP31" s="22"/>
-      <c r="AQ31" s="22"/>
+      <c r="AO31" s="36"/>
+      <c r="AP31" s="21"/>
+      <c r="AQ31" s="21"/>
     </row>
     <row r="32" spans="1:43" ht="17" customHeight="1">
       <c r="A32" s="9">
@@ -2713,9 +2713,9 @@
       <c r="AL32" s="12"/>
       <c r="AM32" s="12"/>
       <c r="AN32" s="13"/>
-      <c r="AO32" s="55"/>
-      <c r="AP32" s="22"/>
-      <c r="AQ32" s="22"/>
+      <c r="AO32" s="36"/>
+      <c r="AP32" s="21"/>
+      <c r="AQ32" s="21"/>
     </row>
     <row r="33" spans="1:43" ht="17" customHeight="1">
       <c r="A33" s="9">
@@ -2760,9 +2760,9 @@
       <c r="AL33" s="12"/>
       <c r="AM33" s="12"/>
       <c r="AN33" s="12"/>
-      <c r="AO33" s="55"/>
-      <c r="AP33" s="22"/>
-      <c r="AQ33" s="22"/>
+      <c r="AO33" s="36"/>
+      <c r="AP33" s="21"/>
+      <c r="AQ33" s="21"/>
     </row>
     <row r="34" spans="1:43" ht="17" customHeight="1">
       <c r="A34" s="9">
@@ -2807,9 +2807,9 @@
       <c r="AL34" s="12"/>
       <c r="AM34" s="12"/>
       <c r="AN34" s="12"/>
-      <c r="AO34" s="56"/>
-      <c r="AP34" s="22"/>
-      <c r="AQ34" s="22"/>
+      <c r="AO34" s="37"/>
+      <c r="AP34" s="21"/>
+      <c r="AQ34" s="21"/>
     </row>
     <row r="35" spans="1:43" ht="17" customHeight="1">
       <c r="A35" s="9">
@@ -2854,170 +2854,142 @@
       <c r="AL35" s="12"/>
       <c r="AM35" s="12"/>
       <c r="AN35" s="13"/>
-      <c r="AO35" s="27" t="s">
+      <c r="AO35" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="AP35" s="22"/>
-      <c r="AQ35" s="22"/>
+      <c r="AP35" s="21"/>
+      <c r="AQ35" s="21"/>
     </row>
     <row r="36" spans="1:43" ht="15" thickBot="1">
       <c r="A36" s="14"/>
-      <c r="B36" s="50" t="s">
+      <c r="B36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="50"/>
-      <c r="D36" s="16">
+      <c r="C36" s="40"/>
+      <c r="D36" s="31">
         <f>SUM(D5:D35)</f>
         <v>0</v>
       </c>
-      <c r="E36" s="50" t="s">
+      <c r="E36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="F36" s="50"/>
-      <c r="G36" s="59">
+      <c r="F36" s="40"/>
+      <c r="G36" s="31">
         <f>SUM(G5:G35)</f>
         <v>0</v>
       </c>
-      <c r="H36" s="50" t="s">
+      <c r="H36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="I36" s="50"/>
-      <c r="J36" s="59">
+      <c r="I36" s="40"/>
+      <c r="J36" s="31">
         <f>SUM(J5:J35)</f>
         <v>0</v>
       </c>
-      <c r="K36" s="50" t="s">
+      <c r="K36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="L36" s="50"/>
+      <c r="L36" s="40"/>
       <c r="M36" s="15">
         <f>SUM(M5:M35)</f>
         <v>0</v>
       </c>
-      <c r="N36" s="50" t="s">
+      <c r="N36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="O36" s="50"/>
+      <c r="O36" s="40"/>
       <c r="P36" s="15">
         <f>SUM(P5:P35)</f>
         <v>0</v>
       </c>
-      <c r="Q36" s="50" t="s">
+      <c r="Q36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="R36" s="50"/>
+      <c r="R36" s="40"/>
       <c r="S36" s="15">
         <f>SUM(S5:S35)</f>
         <v>0</v>
       </c>
-      <c r="T36" s="50" t="s">
+      <c r="T36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="U36" s="50"/>
+      <c r="U36" s="40"/>
       <c r="V36" s="15">
         <f>SUM(V5:V35)</f>
         <v>0</v>
       </c>
-      <c r="W36" s="50" t="s">
+      <c r="W36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="X36" s="50"/>
+      <c r="X36" s="40"/>
       <c r="Y36" s="15">
         <f>SUM(Y5:Y35)</f>
         <v>0</v>
       </c>
-      <c r="Z36" s="50" t="s">
+      <c r="Z36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="AA36" s="50"/>
+      <c r="AA36" s="40"/>
       <c r="AB36" s="15">
         <f>SUM(AB5:AB35)</f>
         <v>0</v>
       </c>
-      <c r="AC36" s="50" t="s">
+      <c r="AC36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="AD36" s="50"/>
+      <c r="AD36" s="40"/>
       <c r="AE36" s="15">
         <f>SUM(AE5:AE35)</f>
         <v>0</v>
       </c>
-      <c r="AF36" s="50" t="s">
+      <c r="AF36" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="AG36" s="50"/>
+      <c r="AG36" s="40"/>
       <c r="AH36" s="15">
         <f>SUM(AH5:AH35)</f>
         <v>0</v>
       </c>
-      <c r="AI36" s="51" t="s">
+      <c r="AI36" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="AJ36" s="51"/>
-      <c r="AK36" s="29">
+      <c r="AJ36" s="32"/>
+      <c r="AK36" s="28">
         <f>SUM(AK5:AK35)</f>
         <v>0</v>
       </c>
-      <c r="AL36" s="57" t="s">
+      <c r="AL36" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="AM36" s="58"/>
-      <c r="AN36" s="10">
+      <c r="AM36" s="39"/>
+      <c r="AN36" s="59">
         <f>SUM(AN5:AN35)</f>
         <v>0</v>
       </c>
-      <c r="AO36" s="28"/>
-      <c r="AP36" s="24"/>
-      <c r="AQ36" s="24"/>
+      <c r="AO36" s="27"/>
+      <c r="AP36" s="23"/>
+      <c r="AQ36" s="23"/>
     </row>
     <row r="37" spans="1:43">
-      <c r="K37" s="17"/>
-      <c r="L37" s="17"/>
-      <c r="M37" s="17"/>
-      <c r="N37" s="17"/>
-      <c r="O37" s="17"/>
-      <c r="P37" s="17"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16"/>
+      <c r="M37" s="16"/>
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
       <c r="T37" s="3"/>
-      <c r="AI37" s="52" t="s">
+      <c r="AI37" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="AJ37" s="52"/>
-      <c r="AK37" s="52"/>
-      <c r="AL37" s="52"/>
-      <c r="AM37" s="52"/>
-      <c r="AN37" s="52"/>
-      <c r="AO37" s="52"/>
+      <c r="AJ37" s="33"/>
+      <c r="AK37" s="33"/>
+      <c r="AL37" s="33"/>
+      <c r="AM37" s="33"/>
+      <c r="AN37" s="33"/>
+      <c r="AO37" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="AI36:AJ36"/>
-    <mergeCell ref="AI37:AO37"/>
-    <mergeCell ref="AO3:AO4"/>
-    <mergeCell ref="AO6:AO13"/>
-    <mergeCell ref="AO17:AO24"/>
-    <mergeCell ref="AO28:AO34"/>
-    <mergeCell ref="AL36:AM36"/>
-    <mergeCell ref="Q36:R36"/>
-    <mergeCell ref="T3:V3"/>
-    <mergeCell ref="T36:U36"/>
-    <mergeCell ref="AF3:AH3"/>
-    <mergeCell ref="AF36:AG36"/>
-    <mergeCell ref="W3:Y3"/>
-    <mergeCell ref="W36:X36"/>
-    <mergeCell ref="Z3:AB3"/>
-    <mergeCell ref="Z36:AA36"/>
-    <mergeCell ref="AC3:AE3"/>
-    <mergeCell ref="AC36:AD36"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="E36:F36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="K36:L36"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="E3:G3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="K3:M3"/>
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="AI1:AJ1"/>
     <mergeCell ref="AN1:AO1"/>
@@ -3030,6 +3002,34 @@
     <mergeCell ref="AK1:AM1"/>
     <mergeCell ref="AK2:AM2"/>
     <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="E3:G3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="E36:F36"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="K36:L36"/>
+    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="Q36:R36"/>
+    <mergeCell ref="T3:V3"/>
+    <mergeCell ref="T36:U36"/>
+    <mergeCell ref="AF3:AH3"/>
+    <mergeCell ref="AF36:AG36"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="W36:X36"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="Z36:AA36"/>
+    <mergeCell ref="AC3:AE3"/>
+    <mergeCell ref="AC36:AD36"/>
+    <mergeCell ref="AI36:AJ36"/>
+    <mergeCell ref="AI37:AO37"/>
+    <mergeCell ref="AO3:AO4"/>
+    <mergeCell ref="AO6:AO13"/>
+    <mergeCell ref="AO17:AO24"/>
+    <mergeCell ref="AO28:AO34"/>
+    <mergeCell ref="AL36:AM36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>